<commit_message>
Add TC-005 Jira bug link
Updated Test_Cases.xlsx with TC-005 negative test result.
Added Jira bug reference KAN-4 for traceability.
</commit_message>
<xml_diff>
--- a/Test_Cases.xlsx
+++ b/Test_Cases.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="39">
   <si>
     <t>Test Case ID</t>
   </si>
@@ -150,12 +150,40 @@
   <si>
     <t>201 Created response returned. Booking was deleted successfully. Get Booking for the same bookingid returned 404 Not Found.</t>
   </si>
+  <si>
+    <t>TC-005</t>
+  </si>
+  <si>
+    <t>Create booking with missing lastname</t>
+  </si>
+  <si>
+    <t>- API/app is accessible.
+- Create Booking request is available in Postman.</t>
+  </si>
+  <si>
+    <t>1. Open Postman and select the Create Booking request.
+2. Remove the firstname field from the request body.
+3. Keep all other required fields valid.
+4. Click Send.</t>
+  </si>
+  <si>
+    <t>- Booking is not created.
+- API returns an error response or validation message.
+- Response does not contain a valid bookingid.</t>
+  </si>
+  <si>
+    <t>Booking was created successfully and response returned a valid bookingid.
+Jira Bug: KAN-4.</t>
+  </si>
+  <si>
+    <t>Failed</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <sz val="11.0"/>
       <color theme="1"/>
@@ -189,8 +217,14 @@
       <color rgb="FF276221"/>
       <name val="Arial"/>
     </font>
+    <font>
+      <b/>
+      <sz val="10.0"/>
+      <color rgb="FFC0504D"/>
+      <name val="Arial"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -215,6 +249,12 @@
         <bgColor rgb="FFC6EFCE"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+        <bgColor rgb="FFFFC7CE"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border/>
@@ -236,7 +276,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -265,6 +305,9 @@
       <alignment readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
     </xf>
     <xf borderId="1" fillId="4" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
+    </xf>
+    <xf borderId="1" fillId="5" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -700,14 +743,28 @@
       <c r="Y5" s="2"/>
       <c r="Z5" s="2"/>
     </row>
-    <row r="6">
-      <c r="A6" s="2"/>
-      <c r="B6" s="2"/>
-      <c r="C6" s="2"/>
-      <c r="D6" s="2"/>
-      <c r="E6" s="2"/>
-      <c r="F6" s="2"/>
-      <c r="G6" s="2"/>
+    <row r="6" ht="122.25" customHeight="1">
+      <c r="A6" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="B6" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="C6" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="D6" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="E6" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="F6" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="G6" s="10" t="s">
+        <v>38</v>
+      </c>
       <c r="H6" s="2"/>
       <c r="I6" s="2"/>
       <c r="J6" s="2"/>

</xml_diff>

<commit_message>
Update negative API test results
Executed TC-006, TC-007, TC-008, and TC-009.
Updated actual results and statuses.
Added Jira bug KAN-5 for failed TC-009.
</commit_message>
<xml_diff>
--- a/Test_Cases.xlsx
+++ b/Test_Cases.xlsx
@@ -9,14 +9,14 @@
   <calcPr/>
   <extLst>
     <ext uri="GoogleSheetsCustomDataVersion2">
-      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId5" roundtripDataChecksum="atLRYru5xsdXdjUglQwQaN4GgYfUkcuRSwX/+pu8bG8="/>
+      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId5" roundtripDataChecksum="rY3PP1X9JHuCz/7j96dg4Q+YAWEdiOf2zdf+uNynTLU="/>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="62">
   <si>
     <t>Test Case ID</t>
   </si>
@@ -162,7 +162,7 @@
   </si>
   <si>
     <t>1. Open Postman and select the Create Booking request.
-2. Remove the firstname field from the request body.
+2. Remove the lastname field from the request body.
 3. Keep all other required fields valid.
 4. Click Send.</t>
   </si>
@@ -177,6 +177,111 @@
   </si>
   <si>
     <t>Failed</t>
+  </si>
+  <si>
+    <t>TC-006</t>
+  </si>
+  <si>
+    <t>Get booking with non-existing booking ID</t>
+  </si>
+  <si>
+    <t>- API/app is accessible.
+- Get Booking request is available in Postman.</t>
+  </si>
+  <si>
+    <t>1. Open Postman and select the Get Booking request.
+2. Set the method to GET.
+3. Enter a booking URL with a non-existing bookingid.
+4. Click Send.</t>
+  </si>
+  <si>
+    <t>- Booking is not found.
+- API returns 404 Not Found or an appropriate error response.
+- Response does not contain booking details.</t>
+  </si>
+  <si>
+    <t>API returned 404 Not Found.
+Response did not contain booking details.</t>
+  </si>
+  <si>
+    <t>TC-007</t>
+  </si>
+  <si>
+    <t>Update booking without token</t>
+  </si>
+  <si>
+    <t>- API/app is accessible.
+- Update Booking request is available in Postman.
+- A valid bookingid exists.</t>
+  </si>
+  <si>
+    <t>1. Open Postman and select the Update Booking request.
+2. Set the method to PUT.
+3. Enter the booking URL with an existing bookingid.
+4. Do not add a valid authentication token.
+5. Enter valid updated booking data in the request body.
+6. Click Send.</t>
+  </si>
+  <si>
+    <t>- Booking is not updated.
+- API returns 403 Forbidden or an authentication error.
+- Response does not show updated booking data.</t>
+  </si>
+  <si>
+    <t>API returned 403 Forbidden.
+Booking was not updated.</t>
+  </si>
+  <si>
+    <t>TC-008</t>
+  </si>
+  <si>
+    <t>Delete booking without token</t>
+  </si>
+  <si>
+    <t>- API/app is accessible.
+- Delete Booking request is available in Postman.
+- A valid bookingid exists.</t>
+  </si>
+  <si>
+    <t>1. Open Postman and select the Delete Booking request.
+2. Set the method to DELETE.
+3. Enter the booking URL with an existing bookingid.
+4. Do not add a valid authentication token.
+5. Click Send.</t>
+  </si>
+  <si>
+    <t>- Booking is not deleted.
+- API returns 403 Forbidden or an authentication error.
+- Booking can still be retrieved by Get Booking.</t>
+  </si>
+  <si>
+    <t>API returned 403 Forbidden.
+Booking was not deleted.</t>
+  </si>
+  <si>
+    <t>TC-009</t>
+  </si>
+  <si>
+    <t>Create booking with invalid checkin date value</t>
+  </si>
+  <si>
+    <t>1. Open Postman and select the Create Booking request.
+2. Set the method to POST.
+3. Fill in all required booking fields with valid data.
+4. Set Check-in Date to "not-a-date".
+5. Keep all other required fields valid.
+6. Click Send.</t>
+  </si>
+  <si>
+    <t>- API returns 400 Bad Request or a validation error.
+- Booking is not created.
+- Response does not contain a valid bookingid.</t>
+  </si>
+  <si>
+    <t>API returned 200 OK.
+Booking was created successfully with invalid checkin date value.
+Response returned a valid bookingid.
+Jira Bug: KAN-5.</t>
   </si>
 </sst>
 </file>
@@ -292,6 +397,9 @@
     <xf borderId="1" fillId="3" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="left" shrinkToFit="0" vertical="top" wrapText="1"/>
     </xf>
+    <xf borderId="1" fillId="3" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
+    </xf>
     <xf borderId="1" fillId="4" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="top" wrapText="1"/>
     </xf>
@@ -299,9 +407,6 @@
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
     </xf>
     <xf borderId="1" fillId="3" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
-    </xf>
-    <xf borderId="1" fillId="3" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
     </xf>
     <xf borderId="1" fillId="4" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
@@ -582,7 +687,7 @@
       <c r="B2" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="C2" s="5" t="s">
         <v>9</v>
       </c>
       <c r="D2" s="4" t="s">
@@ -594,7 +699,7 @@
       <c r="F2" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="G2" s="5" t="s">
+      <c r="G2" s="6" t="s">
         <v>13</v>
       </c>
       <c r="H2" s="2"/>
@@ -618,25 +723,25 @@
       <c r="Z2" s="2"/>
     </row>
     <row r="3" ht="122.25" customHeight="1">
-      <c r="A3" s="6" t="s">
+      <c r="A3" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="B3" s="7" t="s">
+      <c r="B3" s="8" t="s">
         <v>15</v>
       </c>
       <c r="C3" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="D3" s="7" t="s">
+      <c r="D3" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="E3" s="7" t="s">
+      <c r="E3" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="F3" s="7" t="s">
+      <c r="F3" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="G3" s="5" t="s">
+      <c r="G3" s="6" t="s">
         <v>13</v>
       </c>
       <c r="H3" s="2"/>
@@ -660,22 +765,22 @@
       <c r="Z3" s="2"/>
     </row>
     <row r="4" ht="122.25" customHeight="1">
-      <c r="A4" s="6" t="s">
+      <c r="A4" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="B4" s="7" t="s">
+      <c r="B4" s="8" t="s">
         <v>21</v>
       </c>
       <c r="C4" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="D4" s="7" t="s">
+      <c r="D4" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="E4" s="7" t="s">
+      <c r="E4" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="F4" s="7" t="s">
+      <c r="F4" s="8" t="s">
         <v>25</v>
       </c>
       <c r="G4" s="9" t="s">
@@ -702,22 +807,22 @@
       <c r="Z4" s="2"/>
     </row>
     <row r="5" ht="122.25" customHeight="1">
-      <c r="A5" s="6" t="s">
+      <c r="A5" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="B5" s="7" t="s">
+      <c r="B5" s="8" t="s">
         <v>27</v>
       </c>
       <c r="C5" s="8" t="s">
         <v>28</v>
       </c>
-      <c r="D5" s="7" t="s">
+      <c r="D5" s="8" t="s">
         <v>29</v>
       </c>
-      <c r="E5" s="7" t="s">
+      <c r="E5" s="8" t="s">
         <v>30</v>
       </c>
-      <c r="F5" s="7" t="s">
+      <c r="F5" s="8" t="s">
         <v>31</v>
       </c>
       <c r="G5" s="9" t="s">
@@ -744,22 +849,22 @@
       <c r="Z5" s="2"/>
     </row>
     <row r="6" ht="122.25" customHeight="1">
-      <c r="A6" s="6" t="s">
+      <c r="A6" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="B6" s="7" t="s">
+      <c r="B6" s="8" t="s">
         <v>33</v>
       </c>
       <c r="C6" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="D6" s="7" t="s">
+      <c r="D6" s="8" t="s">
         <v>35</v>
       </c>
-      <c r="E6" s="7" t="s">
+      <c r="E6" s="8" t="s">
         <v>36</v>
       </c>
-      <c r="F6" s="7" t="s">
+      <c r="F6" s="8" t="s">
         <v>37</v>
       </c>
       <c r="G6" s="10" t="s">
@@ -785,14 +890,28 @@
       <c r="Y6" s="2"/>
       <c r="Z6" s="2"/>
     </row>
-    <row r="7">
-      <c r="A7" s="2"/>
-      <c r="B7" s="2"/>
-      <c r="C7" s="2"/>
-      <c r="D7" s="2"/>
-      <c r="E7" s="2"/>
-      <c r="F7" s="2"/>
-      <c r="G7" s="2"/>
+    <row r="7" ht="122.25" customHeight="1">
+      <c r="A7" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="B7" s="8" t="s">
+        <v>40</v>
+      </c>
+      <c r="C7" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="D7" s="8" t="s">
+        <v>42</v>
+      </c>
+      <c r="E7" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="F7" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="G7" s="9" t="s">
+        <v>13</v>
+      </c>
       <c r="H7" s="2"/>
       <c r="I7" s="2"/>
       <c r="J7" s="2"/>
@@ -813,14 +932,28 @@
       <c r="Y7" s="2"/>
       <c r="Z7" s="2"/>
     </row>
-    <row r="8">
-      <c r="A8" s="2"/>
-      <c r="B8" s="2"/>
-      <c r="C8" s="2"/>
-      <c r="D8" s="2"/>
-      <c r="E8" s="2"/>
-      <c r="F8" s="2"/>
-      <c r="G8" s="2"/>
+    <row r="8" ht="122.25" customHeight="1">
+      <c r="A8" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="B8" s="8" t="s">
+        <v>46</v>
+      </c>
+      <c r="C8" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="D8" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="E8" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="F8" s="8" t="s">
+        <v>50</v>
+      </c>
+      <c r="G8" s="9" t="s">
+        <v>13</v>
+      </c>
       <c r="H8" s="2"/>
       <c r="I8" s="2"/>
       <c r="J8" s="2"/>
@@ -841,14 +974,28 @@
       <c r="Y8" s="2"/>
       <c r="Z8" s="2"/>
     </row>
-    <row r="9">
-      <c r="A9" s="2"/>
-      <c r="B9" s="2"/>
-      <c r="C9" s="2"/>
-      <c r="D9" s="2"/>
-      <c r="E9" s="2"/>
-      <c r="F9" s="2"/>
-      <c r="G9" s="2"/>
+    <row r="9" ht="122.25" customHeight="1">
+      <c r="A9" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="B9" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="C9" s="8" t="s">
+        <v>53</v>
+      </c>
+      <c r="D9" s="8" t="s">
+        <v>54</v>
+      </c>
+      <c r="E9" s="8" t="s">
+        <v>55</v>
+      </c>
+      <c r="F9" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="G9" s="9" t="s">
+        <v>13</v>
+      </c>
       <c r="H9" s="2"/>
       <c r="I9" s="2"/>
       <c r="J9" s="2"/>
@@ -869,14 +1016,28 @@
       <c r="Y9" s="2"/>
       <c r="Z9" s="2"/>
     </row>
-    <row r="10">
-      <c r="A10" s="2"/>
-      <c r="B10" s="2"/>
-      <c r="C10" s="2"/>
-      <c r="D10" s="2"/>
-      <c r="E10" s="2"/>
-      <c r="F10" s="2"/>
-      <c r="G10" s="2"/>
+    <row r="10" ht="122.25" customHeight="1">
+      <c r="A10" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="B10" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="C10" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="D10" s="8" t="s">
+        <v>59</v>
+      </c>
+      <c r="E10" s="8" t="s">
+        <v>60</v>
+      </c>
+      <c r="F10" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="G10" s="10" t="s">
+        <v>38</v>
+      </c>
       <c r="H10" s="2"/>
       <c r="I10" s="2"/>
       <c r="J10" s="2"/>
@@ -1093,7 +1254,7 @@
       <c r="Y17" s="2"/>
       <c r="Z17" s="2"/>
     </row>
-    <row r="18">
+    <row r="18" ht="15.75" customHeight="1">
       <c r="A18" s="2"/>
       <c r="B18" s="2"/>
       <c r="C18" s="2"/>
@@ -1121,7 +1282,7 @@
       <c r="Y18" s="2"/>
       <c r="Z18" s="2"/>
     </row>
-    <row r="19">
+    <row r="19" ht="15.75" customHeight="1">
       <c r="A19" s="2"/>
       <c r="B19" s="2"/>
       <c r="C19" s="2"/>
@@ -28533,62 +28694,6 @@
       <c r="Y997" s="2"/>
       <c r="Z997" s="2"/>
     </row>
-    <row r="998" ht="15.75" customHeight="1">
-      <c r="A998" s="2"/>
-      <c r="B998" s="2"/>
-      <c r="C998" s="2"/>
-      <c r="D998" s="2"/>
-      <c r="E998" s="2"/>
-      <c r="F998" s="2"/>
-      <c r="G998" s="2"/>
-      <c r="H998" s="2"/>
-      <c r="I998" s="2"/>
-      <c r="J998" s="2"/>
-      <c r="K998" s="2"/>
-      <c r="L998" s="2"/>
-      <c r="M998" s="2"/>
-      <c r="N998" s="2"/>
-      <c r="O998" s="2"/>
-      <c r="P998" s="2"/>
-      <c r="Q998" s="2"/>
-      <c r="R998" s="2"/>
-      <c r="S998" s="2"/>
-      <c r="T998" s="2"/>
-      <c r="U998" s="2"/>
-      <c r="V998" s="2"/>
-      <c r="W998" s="2"/>
-      <c r="X998" s="2"/>
-      <c r="Y998" s="2"/>
-      <c r="Z998" s="2"/>
-    </row>
-    <row r="999" ht="15.75" customHeight="1">
-      <c r="A999" s="2"/>
-      <c r="B999" s="2"/>
-      <c r="C999" s="2"/>
-      <c r="D999" s="2"/>
-      <c r="E999" s="2"/>
-      <c r="F999" s="2"/>
-      <c r="G999" s="2"/>
-      <c r="H999" s="2"/>
-      <c r="I999" s="2"/>
-      <c r="J999" s="2"/>
-      <c r="K999" s="2"/>
-      <c r="L999" s="2"/>
-      <c r="M999" s="2"/>
-      <c r="N999" s="2"/>
-      <c r="O999" s="2"/>
-      <c r="P999" s="2"/>
-      <c r="Q999" s="2"/>
-      <c r="R999" s="2"/>
-      <c r="S999" s="2"/>
-      <c r="T999" s="2"/>
-      <c r="U999" s="2"/>
-      <c r="V999" s="2"/>
-      <c r="W999" s="2"/>
-      <c r="X999" s="2"/>
-      <c r="Y999" s="2"/>
-      <c r="Z999" s="2"/>
-    </row>
   </sheetData>
   <printOptions/>
   <pageMargins bottom="1.0" footer="0.0" header="0.0" left="0.75" right="0.75" top="1.0"/>

</xml_diff>

<commit_message>
Update Batch 2 test results
Executed TC-010 to TC-014.
Updated actual results and statuses.
Linked failed test cases to Jira bugs KAN-6 to KAN-9.
</commit_message>
<xml_diff>
--- a/Test_Cases.xlsx
+++ b/Test_Cases.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="82">
   <si>
     <t>Test Case ID</t>
   </si>
@@ -282,6 +282,97 @@
 Booking was created successfully with invalid checkin date value.
 Response returned a valid bookingid.
 Jira Bug: KAN-5.</t>
+  </si>
+  <si>
+    <t>TC-010</t>
+  </si>
+  <si>
+    <t>Create booking with missing checkin date</t>
+  </si>
+  <si>
+    <t>1. Open Postman and select the Create Booking request.
+2. Remove the checkin date from the request body.
+3. Keep all other required fields valid.
+4. Click Send.</t>
+  </si>
+  <si>
+    <t>API returned 500 Internal Server Error.
+Booking was not created.
+No bookingid was returned.
+Jira Bug: KAN-5</t>
+  </si>
+  <si>
+    <t>TC-011</t>
+  </si>
+  <si>
+    <t>Create booking with missing checkout date</t>
+  </si>
+  <si>
+    <t>1. Open Postman and select the Create Booking request.
+2. Remove the checkout date from the request body.
+3. Keep all other required fields valid.
+4. Click Send.</t>
+  </si>
+  <si>
+    <t>API returned 500 Internal Server Error.
+Booking was not created.
+No bookingid was returned.
+Jira Bug: KAN-6</t>
+  </si>
+  <si>
+    <t>TC-012</t>
+  </si>
+  <si>
+    <t>Create booking with checkout before checkin</t>
+  </si>
+  <si>
+    <t>1. Open Postman and select the Create Booking request.
+2. Set checkin date to 2025-06-10.
+3. Set checkout date to 2025-06-01.
+4. Keep all other required fields valid.
+5. Click Send.</t>
+  </si>
+  <si>
+    <t>API returned 200 OK.
+Booking was created successfully with checkout date before checkin date.
+Response returned a valid bookingid.
+Jira Bug: KAN-7</t>
+  </si>
+  <si>
+    <t>TC-013</t>
+  </si>
+  <si>
+    <t>Create booking with negative total price</t>
+  </si>
+  <si>
+    <t>1. Open Postman and select the Create Booking request.
+2. Set totalprice to -100.
+3. Keep all other required fields valid.
+4. Click Send.</t>
+  </si>
+  <si>
+    <t>API returned 200 OK.
+Booking was created successfully with negative total price.
+Response returned a valid bookingid.
+Jira Bug: KAN-8</t>
+  </si>
+  <si>
+    <t>TC-014</t>
+  </si>
+  <si>
+    <t>Create booking with empty firstname</t>
+  </si>
+  <si>
+    <t>1. Open Postman and select the Create Booking request.
+2. Set firstname to an empty string.
+3. Keep all other required fields valid.
+4. Click Send.</t>
+  </si>
+  <si>
+    <t>API returned 200 OK.
+Booking was created successfully with empty firstname.
+Response returned a valid bookingid.
+Jira Bug: KAN-9</t>
   </si>
 </sst>
 </file>
@@ -1058,14 +1149,28 @@
       <c r="Y10" s="2"/>
       <c r="Z10" s="2"/>
     </row>
-    <row r="11">
-      <c r="A11" s="2"/>
-      <c r="B11" s="2"/>
-      <c r="C11" s="2"/>
-      <c r="D11" s="2"/>
-      <c r="E11" s="2"/>
-      <c r="F11" s="2"/>
-      <c r="G11" s="2"/>
+    <row r="11" ht="122.25" customHeight="1">
+      <c r="A11" s="7" t="s">
+        <v>62</v>
+      </c>
+      <c r="B11" s="8" t="s">
+        <v>63</v>
+      </c>
+      <c r="C11" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="D11" s="8" t="s">
+        <v>64</v>
+      </c>
+      <c r="E11" s="8" t="s">
+        <v>60</v>
+      </c>
+      <c r="F11" s="8" t="s">
+        <v>65</v>
+      </c>
+      <c r="G11" s="10" t="s">
+        <v>38</v>
+      </c>
       <c r="H11" s="2"/>
       <c r="I11" s="2"/>
       <c r="J11" s="2"/>
@@ -1086,14 +1191,28 @@
       <c r="Y11" s="2"/>
       <c r="Z11" s="2"/>
     </row>
-    <row r="12">
-      <c r="A12" s="2"/>
-      <c r="B12" s="2"/>
-      <c r="C12" s="2"/>
-      <c r="D12" s="2"/>
-      <c r="E12" s="2"/>
-      <c r="F12" s="2"/>
-      <c r="G12" s="2"/>
+    <row r="12" ht="122.25" customHeight="1">
+      <c r="A12" s="7" t="s">
+        <v>66</v>
+      </c>
+      <c r="B12" s="8" t="s">
+        <v>67</v>
+      </c>
+      <c r="C12" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="D12" s="8" t="s">
+        <v>68</v>
+      </c>
+      <c r="E12" s="8" t="s">
+        <v>60</v>
+      </c>
+      <c r="F12" s="8" t="s">
+        <v>69</v>
+      </c>
+      <c r="G12" s="10" t="s">
+        <v>38</v>
+      </c>
       <c r="H12" s="2"/>
       <c r="I12" s="2"/>
       <c r="J12" s="2"/>
@@ -1114,14 +1233,28 @@
       <c r="Y12" s="2"/>
       <c r="Z12" s="2"/>
     </row>
-    <row r="13">
-      <c r="A13" s="2"/>
-      <c r="B13" s="2"/>
-      <c r="C13" s="2"/>
-      <c r="D13" s="2"/>
-      <c r="E13" s="2"/>
-      <c r="F13" s="2"/>
-      <c r="G13" s="2"/>
+    <row r="13" ht="122.25" customHeight="1">
+      <c r="A13" s="7" t="s">
+        <v>70</v>
+      </c>
+      <c r="B13" s="8" t="s">
+        <v>71</v>
+      </c>
+      <c r="C13" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="D13" s="8" t="s">
+        <v>72</v>
+      </c>
+      <c r="E13" s="8" t="s">
+        <v>60</v>
+      </c>
+      <c r="F13" s="8" t="s">
+        <v>73</v>
+      </c>
+      <c r="G13" s="10" t="s">
+        <v>38</v>
+      </c>
       <c r="H13" s="2"/>
       <c r="I13" s="2"/>
       <c r="J13" s="2"/>
@@ -1142,14 +1275,28 @@
       <c r="Y13" s="2"/>
       <c r="Z13" s="2"/>
     </row>
-    <row r="14">
-      <c r="A14" s="2"/>
-      <c r="B14" s="2"/>
-      <c r="C14" s="2"/>
-      <c r="D14" s="2"/>
-      <c r="E14" s="2"/>
-      <c r="F14" s="2"/>
-      <c r="G14" s="2"/>
+    <row r="14" ht="122.25" customHeight="1">
+      <c r="A14" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="B14" s="8" t="s">
+        <v>75</v>
+      </c>
+      <c r="C14" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="D14" s="8" t="s">
+        <v>76</v>
+      </c>
+      <c r="E14" s="8" t="s">
+        <v>60</v>
+      </c>
+      <c r="F14" s="8" t="s">
+        <v>77</v>
+      </c>
+      <c r="G14" s="10" t="s">
+        <v>38</v>
+      </c>
       <c r="H14" s="2"/>
       <c r="I14" s="2"/>
       <c r="J14" s="2"/>
@@ -1170,14 +1317,28 @@
       <c r="Y14" s="2"/>
       <c r="Z14" s="2"/>
     </row>
-    <row r="15">
-      <c r="A15" s="2"/>
-      <c r="B15" s="2"/>
-      <c r="C15" s="2"/>
-      <c r="D15" s="2"/>
-      <c r="E15" s="2"/>
-      <c r="F15" s="2"/>
-      <c r="G15" s="2"/>
+    <row r="15" ht="122.25" customHeight="1">
+      <c r="A15" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="B15" s="8" t="s">
+        <v>79</v>
+      </c>
+      <c r="C15" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="D15" s="8" t="s">
+        <v>80</v>
+      </c>
+      <c r="E15" s="8" t="s">
+        <v>60</v>
+      </c>
+      <c r="F15" s="8" t="s">
+        <v>81</v>
+      </c>
+      <c r="G15" s="10" t="s">
+        <v>38</v>
+      </c>
       <c r="H15" s="2"/>
       <c r="I15" s="2"/>
       <c r="J15" s="2"/>

</xml_diff>

<commit_message>
Update test cases to 30 total
Added and executed TC-020 to TC-030.
Updated actual results, statuses, and Jira bug traceability.
Reached 30 total executed test cases.
</commit_message>
<xml_diff>
--- a/Test_Cases.xlsx
+++ b/Test_Cases.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="160" uniqueCount="114">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="248" uniqueCount="175">
   <si>
     <t>Test Case ID</t>
   </si>
@@ -135,9 +135,10 @@
     <t>Delete booking by ID</t>
   </si>
   <si>
-    <t>A valid booking exists.
-A valid bookingid exsists.
-A valid authentication token exsists.</t>
+    <t>- API/app is accessible.
+- A valid bookingid exists.
+- A valid authentication token exists.
+- Delete Booking request is available in Postman.</t>
   </si>
   <si>
     <t>1. Open Postman and select the Delete Booking request.
@@ -460,6 +461,12 @@
     <t>Get booking after delete</t>
   </si>
   <si>
+    <t>- API/app is accessible.
+- Create Booking request is available in Postman.
+- Delete Booking request is available in Postman.
+- A valid authentication token is available.</t>
+  </si>
+  <si>
     <t>1. Create a new booking using POST /booking
 2. Save the bookingid from the response
 3. Create an auth token using POST /auth
@@ -482,6 +489,12 @@
     <t>Update booking with invalid token</t>
   </si>
   <si>
+    <t>- API/app is accessible.
+- Update Booking request is available in Postman.
+- A valid bookingid exists.
+- An invalid authentication token is available.</t>
+  </si>
+  <si>
     <t>1. Open Postman and select the Update Booking request.
 2. Set the method to PUT.
 3. Enter the booking URL with an existing bookingid.
@@ -496,6 +509,250 @@
   <si>
     <t>- API returned 403 Forbidden.
 - Booking was not updated with invalid token.</t>
+  </si>
+  <si>
+    <t>TC-020</t>
+  </si>
+  <si>
+    <t>Delete already deleted booking</t>
+  </si>
+  <si>
+    <t>- API/app is accessible.
+- Create Booking request is available in Postman.
+- Delete Booking request is available in Postman.
+- A valid bookingid exists.
+- A valid authentication token is available.</t>
+  </si>
+  <si>
+    <t>1. Delete an existing booking using DELETE /booking/{id} with a valid token.
+2. Send the same DELETE /booking/{id} request again for the already deleted booking.
+3. Check the response status code and response body.</t>
+  </si>
+  <si>
+    <t>- API returns 404 Not Found or a clear error message.
+- Already deleted booking is not deleted again.</t>
+  </si>
+  <si>
+    <t>- API returned 405 Method Not Allowed.
+- Already deleted booking was not deleted again.</t>
+  </si>
+  <si>
+    <t>TC-021</t>
+  </si>
+  <si>
+    <t>Update non-existing booking ID</t>
+  </si>
+  <si>
+    <t>- API/app is accessible.
+- Update Booking request is available in Postman.
+- A valid authentication token is available.
+- A non-existing bookingid is available.</t>
+  </si>
+  <si>
+    <t>1. Send PUT /booking/{id} request using a non-existing bookingid.
+2. Add a valid authentication token.
+3. Enter valid booking data in the request body.
+4. Send the request.
+5. Check the response status code and response body.</t>
+  </si>
+  <si>
+    <t>- API returns 404 Not Found or a clear error message.
+- Booking is not updated.</t>
+  </si>
+  <si>
+    <t>- API returned 405 Method Not Allowed.
+- Booking was not updated for non-existing bookingid.</t>
+  </si>
+  <si>
+    <t>TC-022</t>
+  </si>
+  <si>
+    <t>Create booking with empty string fields</t>
+  </si>
+  <si>
+    <t>1. Send POST /booking request.
+2. Set firstname, lastname, and additionalneeds as empty strings.
+3. Keep all other required fields valid.
+4. Send the request.
+5. Check the response status code and response body.</t>
+  </si>
+  <si>
+    <t>- API returned 200 OK.
+- Booking was created successfully with empty string fields.
+- Response returned a valid bookingid.</t>
+  </si>
+  <si>
+    <t>KAN-14</t>
+  </si>
+  <si>
+    <t>TC-023</t>
+  </si>
+  <si>
+    <t>Invalid HTTP method on booking endpoint</t>
+  </si>
+  <si>
+    <t>- API/app is accessible.
+- Booking endpoint is available in Postman.</t>
+  </si>
+  <si>
+    <t>1. Send PATCH /booking request without bookingid.
+2. Check the response status code and response body.</t>
+  </si>
+  <si>
+    <t>- API returns 404 Not Found, 405 Method Not Allowed, or a clear error message.
+- Request is not processed successfully.</t>
+  </si>
+  <si>
+    <t>- API returned 404 Not Found.
+- Request was not processed successfully.</t>
+  </si>
+  <si>
+    <t>TC-024</t>
+  </si>
+  <si>
+    <t>Boundary value for total price</t>
+  </si>
+  <si>
+    <t>1. Send POST /booking request.
+2. Set totalprice to 0.
+3. Keep all other required fields valid.
+4. Send the request.
+5. Check the response status code and response body.</t>
+  </si>
+  <si>
+    <t>- API returned 200 OK.
+- Booking was created successfully with totalprice value 0.
+- Response returned a valid bookingid.</t>
+  </si>
+  <si>
+    <t>KAN-15</t>
+  </si>
+  <si>
+    <t>TC-025</t>
+  </si>
+  <si>
+    <t>Create booking with missing totalprice</t>
+  </si>
+  <si>
+    <t>1. Send POST /booking request.
+2. Remove the totalprice field from the request body.
+3. Keep all other required fields valid.
+4. Send the request.
+5. Check the response status code and response body.</t>
+  </si>
+  <si>
+    <t>- API returned 500 Internal Server Error.
+- Booking was not created.
+- No bookingid was returned.</t>
+  </si>
+  <si>
+    <t>KAN-16</t>
+  </si>
+  <si>
+    <t>TC-026</t>
+  </si>
+  <si>
+    <t>Create booking with missing depositpaid</t>
+  </si>
+  <si>
+    <t>1. Send POST /booking request.
+2. Remove the depositpaid field from the request body.
+3. Keep all other required fields valid.
+4. Send the request.
+5. Check the response status code and response body.</t>
+  </si>
+  <si>
+    <t>KAN-17</t>
+  </si>
+  <si>
+    <t>TC-027</t>
+  </si>
+  <si>
+    <t>Create booking with invalid depositpaid value</t>
+  </si>
+  <si>
+    <t>1. Send POST /booking request.
+2. Set depositpaid to an invalid value: "yes".
+3. Keep all other required fields valid.
+4. Send the request.
+5. Check the response status code and response body.</t>
+  </si>
+  <si>
+    <t>- API returned 200 OK.
+- Booking was created successfully with invalid depositpaid value.
+- Response returned a valid bookingid.</t>
+  </si>
+  <si>
+    <t>KAN-18</t>
+  </si>
+  <si>
+    <t>TC-028</t>
+  </si>
+  <si>
+    <t>Get booking with invalid booking ID format</t>
+  </si>
+  <si>
+    <t>1. Send GET /booking/abc request.
+2. Check the response status code and response body.</t>
+  </si>
+  <si>
+    <t>- API returns 404 Not Found, 400 Bad Request, or a clear error message.
+- Booking details are not returned.</t>
+  </si>
+  <si>
+    <t>- API returned 404 Not Found.
+- Booking details were not returned for invalid bookingid format.</t>
+  </si>
+  <si>
+    <t>TC-029</t>
+  </si>
+  <si>
+    <t>Update booking with missing request body</t>
+  </si>
+  <si>
+    <t>- API/app is accessible.
+- Update Booking request is available in Postman.
+- A valid bookingid exists.
+- A valid authentication token is available.</t>
+  </si>
+  <si>
+    <t>1. Send PUT /booking/{id} request with a valid bookingid.
+2. Add a valid authentication token.
+3. Remove the request body.
+4. Send the request.
+5. Check the response status code and response body.</t>
+  </si>
+  <si>
+    <t>- API returns 400 Bad Request or a validation error.
+- Booking is not updated.</t>
+  </si>
+  <si>
+    <t>- API returned 400 Bad Request.
+- Booking was not updated with missing request body.</t>
+  </si>
+  <si>
+    <t>TC-030</t>
+  </si>
+  <si>
+    <t>Delete booking with invalid booking ID format</t>
+  </si>
+  <si>
+    <t>- API/app is accessible.
+- Delete Booking request is available in Postman.
+- A valid authentication token is available.</t>
+  </si>
+  <si>
+    <t>1. Send DELETE /booking/abc request.
+2. Add a valid authentication token.
+3. Check the response status code and response body.</t>
+  </si>
+  <si>
+    <t>- API returns 404 Not Found, 400 Bad Request, or a clear error message.
+- Booking is not deleted.</t>
+  </si>
+  <si>
+    <t>- API returned 405 Method Not Allowed.
+- Booking was not deleted for invalid bookingid format.</t>
   </si>
 </sst>
 </file>
@@ -1680,16 +1937,16 @@
         <v>105</v>
       </c>
       <c r="C19" s="10" t="s">
-        <v>36</v>
+        <v>106</v>
       </c>
       <c r="D19" s="10" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="E19" s="10" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="F19" s="10" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="G19" s="11" t="s">
         <v>14</v>
@@ -1719,22 +1976,22 @@
     </row>
     <row r="20" ht="122.25" customHeight="1">
       <c r="A20" s="9" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B20" s="10" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="C20" s="10" t="s">
-        <v>36</v>
+        <v>112</v>
       </c>
       <c r="D20" s="10" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="E20" s="10" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="F20" s="10" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="G20" s="11" t="s">
         <v>14</v>
@@ -1762,15 +2019,31 @@
       <c r="Z20" s="3"/>
       <c r="AA20" s="3"/>
     </row>
-    <row r="21" ht="15.75" customHeight="1">
-      <c r="A21" s="3"/>
-      <c r="B21" s="3"/>
-      <c r="C21" s="3"/>
-      <c r="D21" s="3"/>
-      <c r="E21" s="3"/>
-      <c r="F21" s="3"/>
-      <c r="G21" s="3"/>
-      <c r="H21" s="13"/>
+    <row r="21" ht="122.25" customHeight="1">
+      <c r="A21" s="9" t="s">
+        <v>116</v>
+      </c>
+      <c r="B21" s="10" t="s">
+        <v>117</v>
+      </c>
+      <c r="C21" s="10" t="s">
+        <v>118</v>
+      </c>
+      <c r="D21" s="10" t="s">
+        <v>119</v>
+      </c>
+      <c r="E21" s="10" t="s">
+        <v>120</v>
+      </c>
+      <c r="F21" s="10" t="s">
+        <v>121</v>
+      </c>
+      <c r="G21" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="H21" s="8" t="s">
+        <v>15</v>
+      </c>
       <c r="I21" s="3"/>
       <c r="J21" s="3"/>
       <c r="K21" s="3"/>
@@ -1791,15 +2064,31 @@
       <c r="Z21" s="3"/>
       <c r="AA21" s="3"/>
     </row>
-    <row r="22" ht="15.75" customHeight="1">
-      <c r="A22" s="3"/>
-      <c r="B22" s="3"/>
-      <c r="C22" s="3"/>
-      <c r="D22" s="3"/>
-      <c r="E22" s="3"/>
-      <c r="F22" s="3"/>
-      <c r="G22" s="3"/>
-      <c r="H22" s="13"/>
+    <row r="22" ht="122.25" customHeight="1">
+      <c r="A22" s="9" t="s">
+        <v>122</v>
+      </c>
+      <c r="B22" s="10" t="s">
+        <v>123</v>
+      </c>
+      <c r="C22" s="10" t="s">
+        <v>124</v>
+      </c>
+      <c r="D22" s="10" t="s">
+        <v>125</v>
+      </c>
+      <c r="E22" s="10" t="s">
+        <v>126</v>
+      </c>
+      <c r="F22" s="10" t="s">
+        <v>127</v>
+      </c>
+      <c r="G22" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="H22" s="8" t="s">
+        <v>15</v>
+      </c>
       <c r="I22" s="3"/>
       <c r="J22" s="3"/>
       <c r="K22" s="3"/>
@@ -1820,15 +2109,31 @@
       <c r="Z22" s="3"/>
       <c r="AA22" s="3"/>
     </row>
-    <row r="23" ht="15.75" customHeight="1">
-      <c r="A23" s="3"/>
-      <c r="B23" s="3"/>
-      <c r="C23" s="3"/>
-      <c r="D23" s="3"/>
-      <c r="E23" s="3"/>
-      <c r="F23" s="3"/>
-      <c r="G23" s="3"/>
-      <c r="H23" s="13"/>
+    <row r="23" ht="122.25" customHeight="1">
+      <c r="A23" s="9" t="s">
+        <v>128</v>
+      </c>
+      <c r="B23" s="10" t="s">
+        <v>129</v>
+      </c>
+      <c r="C23" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="D23" s="10" t="s">
+        <v>130</v>
+      </c>
+      <c r="E23" s="10" t="s">
+        <v>63</v>
+      </c>
+      <c r="F23" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="G23" s="12" t="s">
+        <v>40</v>
+      </c>
+      <c r="H23" s="8" t="s">
+        <v>132</v>
+      </c>
       <c r="I23" s="3"/>
       <c r="J23" s="3"/>
       <c r="K23" s="3"/>
@@ -1849,15 +2154,31 @@
       <c r="Z23" s="3"/>
       <c r="AA23" s="3"/>
     </row>
-    <row r="24" ht="15.75" customHeight="1">
-      <c r="A24" s="3"/>
-      <c r="B24" s="3"/>
-      <c r="C24" s="3"/>
-      <c r="D24" s="3"/>
-      <c r="E24" s="3"/>
-      <c r="F24" s="3"/>
-      <c r="G24" s="3"/>
-      <c r="H24" s="13"/>
+    <row r="24" ht="122.25" customHeight="1">
+      <c r="A24" s="9" t="s">
+        <v>133</v>
+      </c>
+      <c r="B24" s="10" t="s">
+        <v>134</v>
+      </c>
+      <c r="C24" s="10" t="s">
+        <v>135</v>
+      </c>
+      <c r="D24" s="10" t="s">
+        <v>136</v>
+      </c>
+      <c r="E24" s="10" t="s">
+        <v>137</v>
+      </c>
+      <c r="F24" s="10" t="s">
+        <v>138</v>
+      </c>
+      <c r="G24" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="H24" s="8" t="s">
+        <v>15</v>
+      </c>
       <c r="I24" s="3"/>
       <c r="J24" s="3"/>
       <c r="K24" s="3"/>
@@ -1878,15 +2199,31 @@
       <c r="Z24" s="3"/>
       <c r="AA24" s="3"/>
     </row>
-    <row r="25" ht="15.75" customHeight="1">
-      <c r="A25" s="3"/>
-      <c r="B25" s="3"/>
-      <c r="C25" s="3"/>
-      <c r="D25" s="3"/>
-      <c r="E25" s="3"/>
-      <c r="F25" s="3"/>
-      <c r="G25" s="3"/>
-      <c r="H25" s="13"/>
+    <row r="25" ht="122.25" customHeight="1">
+      <c r="A25" s="9" t="s">
+        <v>139</v>
+      </c>
+      <c r="B25" s="10" t="s">
+        <v>140</v>
+      </c>
+      <c r="C25" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="D25" s="10" t="s">
+        <v>141</v>
+      </c>
+      <c r="E25" s="10" t="s">
+        <v>63</v>
+      </c>
+      <c r="F25" s="10" t="s">
+        <v>142</v>
+      </c>
+      <c r="G25" s="12" t="s">
+        <v>40</v>
+      </c>
+      <c r="H25" s="8" t="s">
+        <v>143</v>
+      </c>
       <c r="I25" s="3"/>
       <c r="J25" s="3"/>
       <c r="K25" s="3"/>
@@ -1907,15 +2244,31 @@
       <c r="Z25" s="3"/>
       <c r="AA25" s="3"/>
     </row>
-    <row r="26" ht="15.75" customHeight="1">
-      <c r="A26" s="3"/>
-      <c r="B26" s="3"/>
-      <c r="C26" s="3"/>
-      <c r="D26" s="3"/>
-      <c r="E26" s="3"/>
-      <c r="F26" s="3"/>
-      <c r="G26" s="3"/>
-      <c r="H26" s="13"/>
+    <row r="26" ht="122.25" customHeight="1">
+      <c r="A26" s="9" t="s">
+        <v>144</v>
+      </c>
+      <c r="B26" s="10" t="s">
+        <v>145</v>
+      </c>
+      <c r="C26" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="D26" s="10" t="s">
+        <v>146</v>
+      </c>
+      <c r="E26" s="10" t="s">
+        <v>63</v>
+      </c>
+      <c r="F26" s="10" t="s">
+        <v>147</v>
+      </c>
+      <c r="G26" s="12" t="s">
+        <v>40</v>
+      </c>
+      <c r="H26" s="8" t="s">
+        <v>148</v>
+      </c>
       <c r="I26" s="3"/>
       <c r="J26" s="3"/>
       <c r="K26" s="3"/>
@@ -1936,15 +2289,31 @@
       <c r="Z26" s="3"/>
       <c r="AA26" s="3"/>
     </row>
-    <row r="27" ht="15.75" customHeight="1">
-      <c r="A27" s="3"/>
-      <c r="B27" s="3"/>
-      <c r="C27" s="3"/>
-      <c r="D27" s="3"/>
-      <c r="E27" s="3"/>
-      <c r="F27" s="3"/>
-      <c r="G27" s="3"/>
-      <c r="H27" s="13"/>
+    <row r="27" ht="122.25" customHeight="1">
+      <c r="A27" s="9" t="s">
+        <v>149</v>
+      </c>
+      <c r="B27" s="10" t="s">
+        <v>150</v>
+      </c>
+      <c r="C27" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="D27" s="10" t="s">
+        <v>151</v>
+      </c>
+      <c r="E27" s="10" t="s">
+        <v>63</v>
+      </c>
+      <c r="F27" s="10" t="s">
+        <v>147</v>
+      </c>
+      <c r="G27" s="12" t="s">
+        <v>40</v>
+      </c>
+      <c r="H27" s="8" t="s">
+        <v>152</v>
+      </c>
       <c r="I27" s="3"/>
       <c r="J27" s="3"/>
       <c r="K27" s="3"/>
@@ -1965,15 +2334,31 @@
       <c r="Z27" s="3"/>
       <c r="AA27" s="3"/>
     </row>
-    <row r="28" ht="15.75" customHeight="1">
-      <c r="A28" s="3"/>
-      <c r="B28" s="3"/>
-      <c r="C28" s="3"/>
-      <c r="D28" s="3"/>
-      <c r="E28" s="3"/>
-      <c r="F28" s="3"/>
-      <c r="G28" s="3"/>
-      <c r="H28" s="13"/>
+    <row r="28" ht="122.25" customHeight="1">
+      <c r="A28" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="B28" s="10" t="s">
+        <v>154</v>
+      </c>
+      <c r="C28" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="D28" s="10" t="s">
+        <v>155</v>
+      </c>
+      <c r="E28" s="10" t="s">
+        <v>63</v>
+      </c>
+      <c r="F28" s="10" t="s">
+        <v>156</v>
+      </c>
+      <c r="G28" s="12" t="s">
+        <v>40</v>
+      </c>
+      <c r="H28" s="8" t="s">
+        <v>157</v>
+      </c>
       <c r="I28" s="3"/>
       <c r="J28" s="3"/>
       <c r="K28" s="3"/>
@@ -1994,15 +2379,31 @@
       <c r="Z28" s="3"/>
       <c r="AA28" s="3"/>
     </row>
-    <row r="29" ht="15.75" customHeight="1">
-      <c r="A29" s="3"/>
-      <c r="B29" s="3"/>
-      <c r="C29" s="3"/>
-      <c r="D29" s="3"/>
-      <c r="E29" s="3"/>
-      <c r="F29" s="3"/>
-      <c r="G29" s="3"/>
-      <c r="H29" s="13"/>
+    <row r="29" ht="122.25" customHeight="1">
+      <c r="A29" s="9" t="s">
+        <v>158</v>
+      </c>
+      <c r="B29" s="10" t="s">
+        <v>159</v>
+      </c>
+      <c r="C29" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="D29" s="10" t="s">
+        <v>160</v>
+      </c>
+      <c r="E29" s="10" t="s">
+        <v>161</v>
+      </c>
+      <c r="F29" s="10" t="s">
+        <v>162</v>
+      </c>
+      <c r="G29" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="H29" s="8" t="s">
+        <v>15</v>
+      </c>
       <c r="I29" s="3"/>
       <c r="J29" s="3"/>
       <c r="K29" s="3"/>
@@ -2023,15 +2424,31 @@
       <c r="Z29" s="3"/>
       <c r="AA29" s="3"/>
     </row>
-    <row r="30" ht="15.75" customHeight="1">
-      <c r="A30" s="3"/>
-      <c r="B30" s="3"/>
-      <c r="C30" s="3"/>
-      <c r="D30" s="3"/>
-      <c r="E30" s="3"/>
-      <c r="F30" s="3"/>
-      <c r="G30" s="3"/>
-      <c r="H30" s="13"/>
+    <row r="30" ht="122.25" customHeight="1">
+      <c r="A30" s="9" t="s">
+        <v>163</v>
+      </c>
+      <c r="B30" s="10" t="s">
+        <v>164</v>
+      </c>
+      <c r="C30" s="10" t="s">
+        <v>165</v>
+      </c>
+      <c r="D30" s="10" t="s">
+        <v>166</v>
+      </c>
+      <c r="E30" s="10" t="s">
+        <v>167</v>
+      </c>
+      <c r="F30" s="10" t="s">
+        <v>168</v>
+      </c>
+      <c r="G30" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="H30" s="8" t="s">
+        <v>15</v>
+      </c>
       <c r="I30" s="3"/>
       <c r="J30" s="3"/>
       <c r="K30" s="3"/>
@@ -2052,15 +2469,31 @@
       <c r="Z30" s="3"/>
       <c r="AA30" s="3"/>
     </row>
-    <row r="31" ht="15.75" customHeight="1">
-      <c r="A31" s="3"/>
-      <c r="B31" s="3"/>
-      <c r="C31" s="3"/>
-      <c r="D31" s="3"/>
-      <c r="E31" s="3"/>
-      <c r="F31" s="3"/>
-      <c r="G31" s="3"/>
-      <c r="H31" s="13"/>
+    <row r="31" ht="122.25" customHeight="1">
+      <c r="A31" s="9" t="s">
+        <v>169</v>
+      </c>
+      <c r="B31" s="10" t="s">
+        <v>170</v>
+      </c>
+      <c r="C31" s="10" t="s">
+        <v>171</v>
+      </c>
+      <c r="D31" s="10" t="s">
+        <v>172</v>
+      </c>
+      <c r="E31" s="10" t="s">
+        <v>173</v>
+      </c>
+      <c r="F31" s="10" t="s">
+        <v>174</v>
+      </c>
+      <c r="G31" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="H31" s="8" t="s">
+        <v>15</v>
+      </c>
       <c r="I31" s="3"/>
       <c r="J31" s="3"/>
       <c r="K31" s="3"/>

</xml_diff>

<commit_message>
Update test cases after final review
</commit_message>
<xml_diff>
--- a/Test_Cases.xlsx
+++ b/Test_Cases.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="248" uniqueCount="175">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="248" uniqueCount="174">
   <si>
     <t>Test Case ID</t>
   </si>
@@ -48,20 +48,19 @@
     <t>Create a new booking with valid data</t>
   </si>
   <si>
-    <t>- API/app is accessible.
-- User has valid credentials (if auth required).
-- No existing booking conflicts.</t>
+    <t>- API is accessible.
+- User has valid credentials/token if authentication is required.</t>
   </si>
   <si>
     <t>1. Open Postman and select the Create Booking request.
-2. Fill in 'First Name': John
-3. Fill in 'Last Name': Doe
-4. Fill in 'Total Price': 150
-5. Set 'Deposit Paid': true
-6. Set 'Check-in Date': 2025-06-01
-7. Set 'Check-out Date': 2025-06-05
-8. Fill in 'Additional Needs': Breakfast
-9. Click Send / send POST /booking request.</t>
+2. Set firstname to John.
+3. Set lastname to Doe.
+4. Set totalprice to 150.
+5. Set depositpaid to true.
+6. Set checkin date to 2025-06-01.
+7. Set checkout date to 2025-06-05.
+8. Set additionalneeds to Breakfast.
+9. Send POST /booking request.</t>
   </si>
   <si>
     <t>- HTTP 200 OK response.
@@ -69,7 +68,7 @@
 - Booking details match the submitted data.</t>
   </si>
   <si>
-    <t>200 OK response returned. Response body included bookingid and booking details.</t>
+    <t>200 OK response returned. Response body included a bookingid and the submitted booking details.</t>
   </si>
   <si>
     <t>Passed</t>
@@ -91,8 +90,8 @@
   <si>
     <t>1. Open Postman and select the Get Booking request.
 2. Set the method to GET.
-3. Enter the booking URL with a valid bookingid.
-4. Click Send.</t>
+3. Enter the endpoint URL with a valid bookingid.
+4. Send GET /booking/{id} request.</t>
   </si>
   <si>
     <t>- HTTP 200 OK response.
@@ -108,17 +107,17 @@
     <t>Update booking with valid data</t>
   </si>
   <si>
-    <t>A booking was created successfully.
-A valid bookingid exists.
-A valid authentication token exists.</t>
+    <t>- A booking was created successfully.
+- A valid bookingid exists.
+- A valid authentication token exists.</t>
   </si>
   <si>
     <t>1. Open Postman and select the Update Booking request.
 2. Set the method to PUT.
-3. Enter the booking URL with a valid bookingid.
+3. Enter the endpoint URL with a valid bookingid.
 4. Add a valid authentication token.
 5. Enter updated booking data in the request body.
-6. Click Send.</t>
+6. Send PUT /booking/{id} request.</t>
   </si>
   <si>
     <t>- HTTP 200 OK response.
@@ -126,7 +125,7 @@
 - Response body shows the updated booking data.</t>
   </si>
   <si>
-    <t>200 OK response returned. Booking details were updated successfully</t>
+    <t>200 OK response returned. Booking details were updated successfully.</t>
   </si>
   <si>
     <t>TC-004</t>
@@ -135,7 +134,7 @@
     <t>Delete booking by ID</t>
   </si>
   <si>
-    <t>- API/app is accessible.
+    <t>- API is accessible.
 - A valid bookingid exists.
 - A valid authentication token exists.
 - Delete Booking request is available in Postman.</t>
@@ -145,7 +144,7 @@
 2. Set the method to DELETE.
 3. Enter the booking URL with a valid bookingid.
 4. Add a valid authentication token to headers.
-5. Click Send.
+5. 5. Send DELETE /booking/{id} request.
 6. Open the Get Booking request.
 7. Try to get the same deleted bookingid.</t>
   </si>
@@ -164,14 +163,14 @@
     <t>Create booking with missing lastname</t>
   </si>
   <si>
-    <t>- API/app is accessible.
+    <t>- API is accessible.
 - Create Booking request is available in Postman.</t>
   </si>
   <si>
     <t>1. Open Postman and select the Create Booking request.
 2. Remove the lastname field from the request body.
 3. Keep all other required fields valid.
-4. Click Send.</t>
+4. Send POST /booking request.</t>
   </si>
   <si>
     <t>- Booking is not created.
@@ -179,8 +178,7 @@
 - Response does not contain a valid bookingid.</t>
   </si>
   <si>
-    <t>Booking was created successfully and response returned a valid bookingid.
-Jira Bug: KAN-4.</t>
+    <t>Booking was created successfully and the response returned a valid bookingid.</t>
   </si>
   <si>
     <t>Failed</t>
@@ -195,14 +193,14 @@
     <t>Get booking with non-existing booking ID</t>
   </si>
   <si>
-    <t>- API/app is accessible.
+    <t>- API is accessible.
 - Get Booking request is available in Postman.</t>
   </si>
   <si>
     <t>1. Open Postman and select the Get Booking request.
 2. Set the method to GET.
 3. Enter a booking URL with a non-existing bookingid.
-4. Click Send.</t>
+4. Send GET /booking/{id} request.</t>
   </si>
   <si>
     <t>- Booking is not found.
@@ -220,7 +218,7 @@
     <t>Update booking without token</t>
   </si>
   <si>
-    <t>- API/app is accessible.
+    <t>- API is accessible.
 - Update Booking request is available in Postman.
 - A valid bookingid exists.</t>
   </si>
@@ -230,7 +228,7 @@
 3. Enter the booking URL with an existing bookingid.
 4. Do not add a valid authentication token.
 5. Enter valid updated booking data in the request body.
-6. Click Send.</t>
+6. Send PUT /booking/{id} request.</t>
   </si>
   <si>
     <t>- Booking is not updated.
@@ -248,7 +246,7 @@
     <t>Delete booking without token</t>
   </si>
   <si>
-    <t>- API/app is accessible.
+    <t>- API is accessible.
 - Delete Booking request is available in Postman.
 - A valid bookingid exists.</t>
   </si>
@@ -257,7 +255,7 @@
 2. Set the method to DELETE.
 3. Enter the booking URL with an existing bookingid.
 4. Do not add a valid authentication token.
-5. Click Send.</t>
+5. Send DELETE /booking/{id} request.</t>
   </si>
   <si>
     <t>- Booking is not deleted.
@@ -277,10 +275,10 @@
   <si>
     <t>1. Open Postman and select the Create Booking request.
 2. Set the method to POST.
-3. Fill in all required booking fields with valid data.
+3. Set all required booking fields with valid data.
 4. Set Check-in Date to "not-a-date".
 5. Keep all other required fields valid.
-6. Click Send.</t>
+6. Send POST /booking request.</t>
   </si>
   <si>
     <t>- API returns 400 Bad Request or a validation error.
@@ -306,7 +304,7 @@
     <t>1. Open Postman and select the Create Booking request.
 2. Remove the checkin date from the request body.
 3. Keep all other required fields valid.
-4. Click Send.</t>
+4. Send POST /booking request.</t>
   </si>
   <si>
     <t xml:space="preserve">API returned 500 Internal Server Error.
@@ -327,7 +325,7 @@
     <t>1. Open Postman and select the Create Booking request.
 2. Remove the checkout date from the request body.
 3. Keep all other required fields valid.
-4. Click Send.</t>
+4. Send POST /booking request.</t>
   </si>
   <si>
     <t>TC-012</t>
@@ -340,7 +338,7 @@
 2. Set checkin date to 2025-06-10.
 3. Set checkout date to 2025-06-01.
 4. Keep all other required fields valid.
-5. Click Send.</t>
+5. Send POST /booking request.</t>
   </si>
   <si>
     <t xml:space="preserve">API returned 200 OK.
@@ -361,7 +359,7 @@
     <t>1. Open Postman and select the Create Booking request.
 2. Set totalprice to -100.
 3. Keep all other required fields valid.
-4. Click Send.</t>
+4. Send POST /booking request.</t>
   </si>
   <si>
     <t xml:space="preserve">API returned 200 OK.
@@ -382,7 +380,7 @@
     <t>1. Open Postman and select the Create Booking request.
 2. Set firstname to an empty string.
 3. Keep all other required fields valid.
-4. Click Send.</t>
+4. Send POST /booking request.</t>
   </si>
   <si>
     <t xml:space="preserve">API returned 200 OK.
@@ -403,7 +401,7 @@
     <t>1. Open Postman and select the Create Booking request.
 2. Set firstname with special characters.
 3. Keep all other required fields valid.
-4. Click Send.</t>
+4. Send POST /booking request.</t>
   </si>
   <si>
     <t>- API returned 200 OK.
@@ -423,7 +421,7 @@
     <t>1. Open Postman and select the Create Booking request.
 2. Enter firstname with more than 100 characters.
 3. Keep all other required fields valid.
-4. Click Send.</t>
+4. Send POST /booking request.</t>
   </si>
   <si>
     <t>- API returned 200 OK.
@@ -440,11 +438,11 @@
     <t>Invalid date format</t>
   </si>
   <si>
-    <t>1. Send POST /booking request
-2. Enter checkin date with invalid format: 30-12-2026
-3. Enter checkout date with valid format: 2026-12-31
-4. Send the request
-5. Check the response status code and response body</t>
+    <t>1. Open Postman and select the Create Booking request.
+2. Enter checkin date with invalid format: 30-12-2026.
+3. Enter checkout date with valid format: 2026-12-31.
+4. Send POST /booking request.
+5. Check the response status code and response body.</t>
   </si>
   <si>
     <t>- API returned 200 OK.
@@ -461,18 +459,18 @@
     <t>Get booking after delete</t>
   </si>
   <si>
-    <t>- API/app is accessible.
+    <t>- API is accessible.
 - Create Booking request is available in Postman.
 - Delete Booking request is available in Postman.
 - A valid authentication token is available.</t>
   </si>
   <si>
-    <t>1. Create a new booking using POST /booking
-2. Save the bookingid from the response
-3. Create an auth token using POST /auth
-4. Delete the booking using DELETE /booking/{id} with a valid token
-5. Send GET /booking/{id} for the deleted booking
-6. Check the response status code and response body</t>
+    <t>1. Create a new booking using POST /booking.
+2. Save the bookingid from the response.
+3. Create an auth token using POST /auth.
+4. Delete the booking using DELETE /booking/{id} with a valid token.
+5. Send GET /booking/{id} for the deleted booking.
+6. Check the response status code and response body.</t>
   </si>
   <si>
     <t>- API returns 404 Not Found.
@@ -489,7 +487,7 @@
     <t>Update booking with invalid token</t>
   </si>
   <si>
-    <t>- API/app is accessible.
+    <t>- API is accessible.
 - Update Booking request is available in Postman.
 - A valid bookingid exists.
 - An invalid authentication token is available.</t>
@@ -500,7 +498,7 @@
 3. Enter the booking URL with an existing bookingid.
 4. Add an invalid authentication token.
 5. Enter valid updated booking data in the request body.
-6. Click Send.</t>
+6. Send PUT /booking/{id} request.</t>
   </si>
   <si>
     <t>- API returns 401 Unauthorized or 403 Forbidden.
@@ -517,7 +515,7 @@
     <t>Delete already deleted booking</t>
   </si>
   <si>
-    <t>- API/app is accessible.
+    <t>- API is accessible.
 - Create Booking request is available in Postman.
 - Delete Booking request is available in Postman.
 - A valid bookingid exists.
@@ -529,7 +527,7 @@
 3. Check the response status code and response body.</t>
   </si>
   <si>
-    <t>- API returns 404 Not Found or a clear error message.
+    <t>- API returns 404 Not Found, 405 Method Not Allowed, or a clear error response.
 - Already deleted booking is not deleted again.</t>
   </si>
   <si>
@@ -543,20 +541,22 @@
     <t>Update non-existing booking ID</t>
   </si>
   <si>
-    <t>- API/app is accessible.
+    <t>- API is accessible.
 - Update Booking request is available in Postman.
 - A valid authentication token is available.
 - A non-existing bookingid is available.</t>
   </si>
   <si>
-    <t>1. Send PUT /booking/{id} request using a non-existing bookingid.
-2. Add a valid authentication token.
-3. Enter valid booking data in the request body.
-4. Send the request.
-5. Check the response status code and response body.</t>
+    <t>1. Open Postman and select the Update Booking request.
+2. Set the method to PUT.
+3. Enter the endpoint URL with a non-existing bookingid.
+4. Add a valid authentication token.
+5. Enter valid booking data in the request body.
+6. Send PUT /booking/{id} request.
+7. Check the response status code and response body.</t>
   </si>
   <si>
-    <t>- API returns 404 Not Found or a clear error message.
+    <t>- API returns 404 Not Found, 405 Method Not Allowed, or a clear error response.
 - Booking is not updated.</t>
   </si>
   <si>
@@ -570,10 +570,10 @@
     <t>Create booking with empty string fields</t>
   </si>
   <si>
-    <t>1. Send POST /booking request.
+    <t>1. Open Postman and select the Create Booking request.
 2. Set firstname, lastname, and additionalneeds as empty strings.
 3. Keep all other required fields valid.
-4. Send the request.
+4. Send POST /booking request.
 5. Check the response status code and response body.</t>
   </si>
   <si>
@@ -591,12 +591,14 @@
     <t>Invalid HTTP method on booking endpoint</t>
   </si>
   <si>
-    <t>- API/app is accessible.
+    <t>- API is accessible.
 - Booking endpoint is available in Postman.</t>
   </si>
   <si>
-    <t>1. Send PATCH /booking request without bookingid.
-2. Check the response status code and response body.</t>
+    <t>1. Open Postman and select the booking endpoint request.
+2. Set the method to PATCH.
+3. Send PATCH /booking request without a bookingid.
+4. Check the response status code and response body.</t>
   </si>
   <si>
     <t>- API returns 404 Not Found, 405 Method Not Allowed, or a clear error message.
@@ -613,10 +615,10 @@
     <t>Boundary value for total price</t>
   </si>
   <si>
-    <t>1. Send POST /booking request.
+    <t>1. Open Postman and select the Create Booking request.
 2. Set totalprice to 0.
 3. Keep all other required fields valid.
-4. Send the request.
+4. Send POST /booking request.
 5. Check the response status code and response body.</t>
   </si>
   <si>
@@ -634,10 +636,10 @@
     <t>Create booking with missing totalprice</t>
   </si>
   <si>
-    <t>1. Send POST /booking request.
+    <t>1. Open Postman and select the Create Booking request.
 2. Remove the totalprice field from the request body.
 3. Keep all other required fields valid.
-4. Send the request.
+4. Send POST /booking request.
 5. Check the response status code and response body.</t>
   </si>
   <si>
@@ -655,10 +657,10 @@
     <t>Create booking with missing depositpaid</t>
   </si>
   <si>
-    <t>1. Send POST /booking request.
+    <t>1. Open Postman and select the Create Booking request.
 2. Remove the depositpaid field from the request body.
 3. Keep all other required fields valid.
-4. Send the request.
+4. Send POST /booking request.
 5. Check the response status code and response body.</t>
   </si>
   <si>
@@ -671,10 +673,10 @@
     <t>Create booking with invalid depositpaid value</t>
   </si>
   <si>
-    <t>1. Send POST /booking request.
-2. Set depositpaid to an invalid value: "yes".
+    <t>1. Open Postman and select the Create Booking request.
+2. Set depositpaid to an invalid value.
 3. Keep all other required fields valid.
-4. Send the request.
+4. Send POST /booking request.
 5. Check the response status code and response body.</t>
   </si>
   <si>
@@ -696,10 +698,6 @@
 2. Check the response status code and response body.</t>
   </si>
   <si>
-    <t>- API returns 404 Not Found, 400 Bad Request, or a clear error message.
-- Booking details are not returned.</t>
-  </si>
-  <si>
     <t>- API returned 404 Not Found.
 - Booking details were not returned for invalid bookingid format.</t>
   </si>
@@ -710,17 +708,19 @@
     <t>Update booking with missing request body</t>
   </si>
   <si>
-    <t>- API/app is accessible.
+    <t>- API is accessible.
 - Update Booking request is available in Postman.
 - A valid bookingid exists.
 - A valid authentication token is available.</t>
   </si>
   <si>
-    <t>1. Send PUT /booking/{id} request with a valid bookingid.
-2. Add a valid authentication token.
-3. Remove the request body.
-4. Send the request.
-5. Check the response status code and response body.</t>
+    <t>1. Open Postman and select the Update Booking request.
+2. Set the method to PUT.
+3. Enter the endpoint URL with a valid bookingid.
+4. Add a valid authentication token.
+5. Remove the request body.
+6. Send PUT /booking/{id} request.
+7. Check the response status code and response body.</t>
   </si>
   <si>
     <t>- API returns 400 Bad Request or a validation error.
@@ -737,17 +737,20 @@
     <t>Delete booking with invalid booking ID format</t>
   </si>
   <si>
-    <t>- API/app is accessible.
+    <t>- API is accessible.
 - Delete Booking request is available in Postman.
 - A valid authentication token is available.</t>
   </si>
   <si>
-    <t>1. Send DELETE /booking/abc request.
-2. Add a valid authentication token.
-3. Check the response status code and response body.</t>
+    <t>1. Open Postman and select the Delete Booking request.
+2. Set the method to DELETE.
+3. Enter the endpoint URL with invalid bookingid format: /booking/abc.
+4. Add a valid authentication token.
+5. Send DELETE /booking/abc request.
+6. Check the response status code and response body.</t>
   </si>
   <si>
-    <t>- API returns 404 Not Found, 400 Bad Request, or a clear error message.
+    <t>- API returns 404 Not Found, 400 Bad Request, 405 Method Not Allowed, or a clear error response.
 - Booking is not deleted.</t>
   </si>
   <si>
@@ -1174,13 +1177,13 @@
       <c r="C2" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="D2" s="5" t="s">
+      <c r="D2" s="6" t="s">
         <v>11</v>
       </c>
       <c r="E2" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="F2" s="5" t="s">
+      <c r="F2" s="6" t="s">
         <v>13</v>
       </c>
       <c r="G2" s="7" t="s">
@@ -2396,7 +2399,7 @@
         <v>161</v>
       </c>
       <c r="F29" s="10" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="G29" s="11" t="s">
         <v>14</v>
@@ -2426,22 +2429,22 @@
     </row>
     <row r="30" ht="122.25" customHeight="1">
       <c r="A30" s="9" t="s">
+        <v>162</v>
+      </c>
+      <c r="B30" s="10" t="s">
         <v>163</v>
       </c>
-      <c r="B30" s="10" t="s">
+      <c r="C30" s="10" t="s">
         <v>164</v>
       </c>
-      <c r="C30" s="10" t="s">
+      <c r="D30" s="10" t="s">
         <v>165</v>
       </c>
-      <c r="D30" s="10" t="s">
+      <c r="E30" s="10" t="s">
         <v>166</v>
       </c>
-      <c r="E30" s="10" t="s">
+      <c r="F30" s="10" t="s">
         <v>167</v>
-      </c>
-      <c r="F30" s="10" t="s">
-        <v>168</v>
       </c>
       <c r="G30" s="11" t="s">
         <v>14</v>
@@ -2471,22 +2474,22 @@
     </row>
     <row r="31" ht="122.25" customHeight="1">
       <c r="A31" s="9" t="s">
+        <v>168</v>
+      </c>
+      <c r="B31" s="10" t="s">
         <v>169</v>
       </c>
-      <c r="B31" s="10" t="s">
+      <c r="C31" s="10" t="s">
         <v>170</v>
       </c>
-      <c r="C31" s="10" t="s">
+      <c r="D31" s="10" t="s">
         <v>171</v>
       </c>
-      <c r="D31" s="10" t="s">
+      <c r="E31" s="10" t="s">
         <v>172</v>
       </c>
-      <c r="E31" s="10" t="s">
+      <c r="F31" s="10" t="s">
         <v>173</v>
-      </c>
-      <c r="F31" s="10" t="s">
-        <v>174</v>
       </c>
       <c r="G31" s="11" t="s">
         <v>14</v>

</xml_diff>